<commit_message>
Kit de teste: Consultoria Aurora (cliente de serviços) e arquivo de apoio ao Enquadramento, com testes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVrp8HXiJ3fo8syeVkDidK
</commit_message>
<xml_diff>
--- a/kit-de-teste/1-clientes-para-importar.xlsx
+++ b/kit-de-teste/1-clientes-para-importar.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -507,20 +507,44 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>00.000.000/0001-91</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>98.765.432/0001-98</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Consultoria Aurora Ltda</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Serviços fator R</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Simples Nacional</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>contato@consultoriaaurora.example</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>(11) 97777-6666</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Seu Álvaro</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>33.000.167/0001-01</t>
+          <t>00.000.000/0001-91</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -533,7 +557,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>47.960.950/0001-21</t>
+          <t>33.000.167/0001-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -546,7 +570,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>07.526.557/0001-00</t>
+          <t>47.960.950/0001-21</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -559,7 +583,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>33.592.510/0001-54</t>
+          <t>07.526.557/0001-00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -572,7 +596,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>71.673.990/0001-77</t>
+          <t>33.592.510/0001-54</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -585,7 +609,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>16.670.085/0001-55</t>
+          <t>71.673.990/0001-77</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -598,24 +622,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>12.345.678/0001-96</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Empresa com CNPJ digitado errado</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Serviços</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>MEI</t>
-        </is>
-      </c>
+          <t>16.670.085/0001-55</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -623,15 +635,40 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>71.673.990/0001-77</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+          <t>12.345.678/0001-96</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Empresa com CNPJ digitado errado</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Serviços</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>71.673.990/0001-77</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>